<commit_message>
motor driver from scratch and 3dp parts update and fixes, features
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\tech\robotyka\robots\evangelion-turbo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6E0C222-BC14-4273-BB21-FD94A1DCA2A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B5CA423-BB99-4669-B6DD-E35BF87614E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="480" windowWidth="38640" windowHeight="21240" xr2:uid="{C42FA279-E8B3-4402-922D-DA72FD085F98}"/>
   </bookViews>
@@ -1622,11 +1622,11 @@
         <v>74</v>
       </c>
       <c r="B30" s="10">
-        <v>1500</v>
+        <v>1000</v>
       </c>
       <c r="C30" s="8">
         <f t="shared" si="0"/>
-        <v>411.97473221642406</v>
+        <v>274.64982147761606</v>
       </c>
       <c r="D30" s="12" t="s">
         <v>75</v>

</xml_diff>

<commit_message>
motor driver update - rethinking about galvanic isolation
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\tech\robotyka\robots\evangelion-turbo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B5CA423-BB99-4669-B6DD-E35BF87614E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CE76245-BF1D-4E57-A912-651F74351069}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="480" windowWidth="38640" windowHeight="21240" xr2:uid="{C42FA279-E8B3-4402-922D-DA72FD085F98}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="76">
   <si>
     <t>banana plug 2mm pair 10pcs</t>
   </si>
@@ -259,15 +259,6 @@
   </si>
   <si>
     <t>for sensors</t>
-  </si>
-  <si>
-    <t>I will rob most of the resistors and capacitors from by brother :)</t>
-  </si>
-  <si>
-    <t>My brother</t>
-  </si>
-  <si>
-    <t>He said it is okay tho :)</t>
   </si>
   <si>
     <t>like MCU, connector, buck conv, MOSFETs… Letme know if anyone need exact BOM here</t>
@@ -1619,7 +1610,7 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="16" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B30" s="10">
         <v>1000</v>
@@ -1629,15 +1620,15 @@
         <v>274.64982147761606</v>
       </c>
       <c r="D30" s="12" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E30" s="17" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="16" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B31" s="10">
         <v>500</v>
@@ -1647,10 +1638,10 @@
         <v>137.32491073880803</v>
       </c>
       <c r="D31" s="12" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E31" s="17" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
@@ -1659,109 +1650,97 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C33" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C34" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C35" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C36" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C37" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C38" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C39" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A40" s="16" t="s">
-        <v>70</v>
-      </c>
-      <c r="B40" s="10">
-        <v>0</v>
-      </c>
+    <row r="40" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C40" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="D40" s="12" t="s">
-        <v>71</v>
-      </c>
-      <c r="E40" s="17" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="41" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C41" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C42" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C43" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C44" s="8">
         <f>#REF!/$H$2</f>
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C45" s="8">
         <f>#REF!/$H$2</f>
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C46" s="8">
         <f>#REF!/$H$2</f>
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C47" s="8">
         <f>#REF!/$H$2</f>
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C48" s="8">
         <f>#REF!/$H$2</f>
         <v>0</v>

</xml_diff>